<commit_message>
mmlu full data run results for tiny aya global
</commit_message>
<xml_diff>
--- a/results/hypothesis_1/mgsm/final_accuracies_mgsm.xlsx
+++ b/results/hypothesis_1/mgsm/final_accuracies_mgsm.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,279 +459,930 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>tiny-aya-earth</t>
+          <t>gemma3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>sw</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.644</v>
+        <v>0.904</v>
       </c>
       <c r="D2" t="n">
-        <v>161</v>
+        <v>226</v>
       </c>
       <c r="E2" t="n">
         <v>250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>final_data_tiny-aya-earth.xlsx</t>
+          <t>final_data_gemma3.xlsx</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>cot_majority_sw</t>
+          <t>cot_majority_en</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>tiny-aya-fire</t>
+          <t>gemma3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>bn</t>
+          <t>zh</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.58</v>
+        <v>0.716</v>
       </c>
       <c r="D3" t="n">
-        <v>145</v>
+        <v>179</v>
       </c>
       <c r="E3" t="n">
         <v>250</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>final_data_tiny-aya-fire.xlsx</t>
+          <t>final_data_gemma3.xlsx</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>cot_majority_bn</t>
+          <t>cot_majority_zh</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>tiny-aya-fire</t>
+          <t>gemma3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>te</t>
+          <t>bn</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.548</v>
+        <v>0.648</v>
       </c>
       <c r="D4" t="n">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="E4" t="n">
         <v>250</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>final_data_tiny-aya-fire.xlsx</t>
+          <t>final_data_gemma3.xlsx</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>cot_majority_te</t>
+          <t>cot_majority_bn</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>gemma3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>en</t>
+          <t>te</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.788</v>
+        <v>0.652</v>
       </c>
       <c r="D5" t="n">
-        <v>197</v>
+        <v>163</v>
       </c>
       <c r="E5" t="n">
         <v>250</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>final_data_tiny-aya-global.xlsx</t>
+          <t>final_data_gemma3.xlsx</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>cot_majority_en</t>
+          <t>cot_majority_te</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>gemma3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>zh</t>
+          <t>sw</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.612</v>
+        <v>0.544</v>
       </c>
       <c r="D6" t="n">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="E6" t="n">
         <v>250</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>final_data_tiny-aya-global.xlsx</t>
+          <t>final_data_gemma3.xlsx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>cot_majority_zh</t>
+          <t>cot_majority_sw</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>qwen3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>bn</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.584</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>146</v>
+        <v>234</v>
       </c>
       <c r="E7" t="n">
         <v>250</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>final_data_tiny-aya-global.xlsx</t>
+          <t>final_data_qwen3.xlsx</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>cot_majority_bn</t>
+          <t>cot_majority_en</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>qwen3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>te</t>
+          <t>zh</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.876</v>
       </c>
       <c r="D8" t="n">
-        <v>140</v>
+        <v>219</v>
       </c>
       <c r="E8" t="n">
         <v>250</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>final_data_tiny-aya-global.xlsx</t>
+          <t>final_data_qwen3.xlsx</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>cot_majority_te</t>
+          <t>cot_majority_zh</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>qwen3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>sw</t>
+          <t>bn</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.588</v>
+        <v>0.712</v>
       </c>
       <c r="D9" t="n">
-        <v>147</v>
+        <v>178</v>
       </c>
       <c r="E9" t="n">
         <v>250</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>final_data_tiny-aya-global.xlsx</t>
+          <t>final_data_qwen3.xlsx</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>cot_majority_sw</t>
+          <t>cot_majority_bn</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>qwen3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="D10" t="n">
+        <v>156</v>
+      </c>
+      <c r="E10" t="n">
+        <v>250</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>final_data_qwen3.xlsx</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>cot_majority_te</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>qwen3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="D11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E11" t="n">
+        <v>250</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>final_data_qwen3.xlsx</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>cot_majority_sw</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>tiny-aya-earth</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.756</v>
+      </c>
+      <c r="D12" t="n">
+        <v>189</v>
+      </c>
+      <c r="E12" t="n">
+        <v>250</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-earth.xlsx</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>cot_majority_en</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>tiny-aya-earth</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.616</v>
+      </c>
+      <c r="D13" t="n">
+        <v>154</v>
+      </c>
+      <c r="E13" t="n">
+        <v>250</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-earth.xlsx</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>cot_majority_zh</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>tiny-aya-earth</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.592</v>
+      </c>
+      <c r="D14" t="n">
+        <v>148</v>
+      </c>
+      <c r="E14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-earth.xlsx</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>cot_majority_bn</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>tiny-aya-earth</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.544</v>
+      </c>
+      <c r="D15" t="n">
+        <v>136</v>
+      </c>
+      <c r="E15" t="n">
+        <v>250</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-earth.xlsx</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>cot_majority_te</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>tiny-aya-earth</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.616</v>
+      </c>
+      <c r="D16" t="n">
+        <v>154</v>
+      </c>
+      <c r="E16" t="n">
+        <v>250</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-earth.xlsx</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>cot_majority_sw</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="D17" t="n">
+        <v>185</v>
+      </c>
+      <c r="E17" t="n">
+        <v>250</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-fire.xlsx</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>cot_majority_en</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="D18" t="n">
+        <v>156</v>
+      </c>
+      <c r="E18" t="n">
+        <v>250</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-fire.xlsx</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>cot_majority_zh</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="D19" t="n">
+        <v>140</v>
+      </c>
+      <c r="E19" t="n">
+        <v>250</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-fire.xlsx</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>cot_majority_bn</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.556</v>
+      </c>
+      <c r="D20" t="n">
+        <v>139</v>
+      </c>
+      <c r="E20" t="n">
+        <v>250</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-fire.xlsx</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>cot_majority_te</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.604</v>
+      </c>
+      <c r="D21" t="n">
+        <v>151</v>
+      </c>
+      <c r="E21" t="n">
+        <v>250</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-fire.xlsx</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>cot_majority_sw</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="D22" t="n">
+        <v>197</v>
+      </c>
+      <c r="E22" t="n">
+        <v>250</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-global.xlsx</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>cot_majority_en</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="D23" t="n">
+        <v>153</v>
+      </c>
+      <c r="E23" t="n">
+        <v>250</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-global.xlsx</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>cot_majority_zh</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.584</v>
+      </c>
+      <c r="D24" t="n">
+        <v>146</v>
+      </c>
+      <c r="E24" t="n">
+        <v>250</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-global.xlsx</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>cot_majority_bn</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="D25" t="n">
+        <v>140</v>
+      </c>
+      <c r="E25" t="n">
+        <v>250</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-global.xlsx</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>cot_majority_te</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.588</v>
+      </c>
+      <c r="D26" t="n">
+        <v>147</v>
+      </c>
+      <c r="E26" t="n">
+        <v>250</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-global.xlsx</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>cot_majority_sw</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>tiny-aya-water</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.752</v>
+      </c>
+      <c r="D27" t="n">
+        <v>188</v>
+      </c>
+      <c r="E27" t="n">
+        <v>250</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-water.xlsx</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>cot_majority_en</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
         <is>
           <t>zh</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D10" t="n">
-        <v>150</v>
-      </c>
-      <c r="E10" t="n">
-        <v>250</v>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="C28" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="D28" t="n">
+        <v>156</v>
+      </c>
+      <c r="E28" t="n">
+        <v>250</v>
+      </c>
+      <c r="F28" t="inlineStr">
         <is>
           <t>final_data_tiny-aya-water.xlsx</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>cot_majority_zh</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="D29" t="n">
+        <v>134</v>
+      </c>
+      <c r="E29" t="n">
+        <v>250</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-water.xlsx</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>cot_majority_bn</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0.556</v>
+      </c>
+      <c r="D30" t="n">
+        <v>139</v>
+      </c>
+      <c r="E30" t="n">
+        <v>250</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-water.xlsx</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>cot_majority_te</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0.608</v>
+      </c>
+      <c r="D31" t="n">
+        <v>152</v>
+      </c>
+      <c r="E31" t="n">
+        <v>250</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>final_data_tiny-aya-water.xlsx</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>cot_majority_sw</t>
         </is>
       </c>
     </row>
@@ -746,7 +1397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -789,7 +1440,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>tiny-aya-earth</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -798,17 +1449,17 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.044</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E2" t="n">
         <v>250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>final_direct_tiny-aya-global.xlsx</t>
+          <t>final_direct_tiny-aya-earth.xlsx</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -820,7 +1471,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>tiny-aya-earth</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -829,17 +1480,17 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.044</v>
+        <v>0.064</v>
       </c>
       <c r="D3" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E3" t="n">
         <v>250</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>final_direct_tiny-aya-global.xlsx</t>
+          <t>final_direct_tiny-aya-earth.xlsx</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -851,7 +1502,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>tiny-aya-earth</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -860,17 +1511,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.052</v>
+        <v>0.044</v>
       </c>
       <c r="D4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E4" t="n">
         <v>250</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>final_direct_tiny-aya-global.xlsx</t>
+          <t>final_direct_tiny-aya-earth.xlsx</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -882,7 +1533,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>tiny-aya-earth</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -891,17 +1542,17 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.048</v>
+        <v>0.044</v>
       </c>
       <c r="D5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E5" t="n">
         <v>250</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>final_direct_tiny-aya-global.xlsx</t>
+          <t>final_direct_tiny-aya-earth.xlsx</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -913,29 +1564,494 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>tiny-aya-earth</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="D6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E6" t="n">
+        <v>250</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-earth.xlsx</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>direct_majority_sw</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="D7" t="n">
+        <v>18</v>
+      </c>
+      <c r="E7" t="n">
+        <v>250</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-fire.xlsx</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>direct_majority_en</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="D8" t="n">
+        <v>17</v>
+      </c>
+      <c r="E8" t="n">
+        <v>250</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-fire.xlsx</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>direct_majority_zh</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="D9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E9" t="n">
+        <v>250</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-fire.xlsx</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>direct_majority_bn</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="D10" t="n">
+        <v>11</v>
+      </c>
+      <c r="E10" t="n">
+        <v>250</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-fire.xlsx</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>direct_majority_te</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="D11" t="n">
+        <v>13</v>
+      </c>
+      <c r="E11" t="n">
+        <v>250</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-fire.xlsx</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>direct_majority_sw</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>tiny-aya-global</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="D12" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" t="n">
+        <v>250</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-global.xlsx</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>direct_majority_en</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="D13" t="n">
+        <v>11</v>
+      </c>
+      <c r="E13" t="n">
+        <v>250</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-global.xlsx</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>direct_majority_zh</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="D14" t="n">
+        <v>13</v>
+      </c>
+      <c r="E14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-global.xlsx</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>direct_majority_bn</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="D15" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" t="n">
+        <v>250</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-global.xlsx</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>direct_majority_te</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>sw</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C16" t="n">
         <v>0.036</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D16" t="n">
         <v>9</v>
       </c>
-      <c r="E6" t="n">
-        <v>250</v>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="E16" t="n">
+        <v>250</v>
+      </c>
+      <c r="F16" t="inlineStr">
         <is>
           <t>final_direct_tiny-aya-global.xlsx</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>direct_majority_sw</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D17" t="n">
+        <v>15</v>
+      </c>
+      <c r="E17" t="n">
+        <v>250</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-water.xlsx</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>direct_majority_en</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E18" t="n">
+        <v>250</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-water.xlsx</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>direct_majority_zh</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="D19" t="n">
+        <v>13</v>
+      </c>
+      <c r="E19" t="n">
+        <v>250</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-water.xlsx</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>direct_majority_bn</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="D20" t="n">
+        <v>9</v>
+      </c>
+      <c r="E20" t="n">
+        <v>250</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-water.xlsx</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>direct_majority_te</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="D21" t="n">
+        <v>13</v>
+      </c>
+      <c r="E21" t="n">
+        <v>250</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>final_direct_tiny-aya-water.xlsx</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
         <is>
           <t>direct_majority_sw</t>
         </is>
@@ -952,7 +2068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -980,7 +2096,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>tiny-aya-earth</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -989,16 +2105,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.744</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7782426778242678</v>
+        <v>0.7370689655172414</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>tiny-aya-earth</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1007,16 +2123,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.552</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5941422594142259</v>
+        <v>0.5897435897435899</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>tiny-aya-earth</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1025,16 +2141,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.5319999999999999</v>
+        <v>0.5479999999999999</v>
       </c>
       <c r="D4" t="n">
-        <v>0.561181434599156</v>
+        <v>0.5732217573221757</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>tiny-aya-earth</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1043,28 +2159,298 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.512</v>
+        <v>0.5</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5378151260504203</v>
+        <v>0.5230125523012552</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>tiny-aya-earth</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.5966386554621849</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.668</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.7198275862068966</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.556</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.5965665236051503</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.512</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.5378151260504203</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.512</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.5355648535564854</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.5519999999999999</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.5822784810126582</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>tiny-aya-global</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.744</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.7782426778242678</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.5941422594142259</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.5319999999999999</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.561181434599156</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.512</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.5378151260504203</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>sw</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C16" t="n">
         <v>0.5519999999999999</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D16" t="n">
         <v>0.5726141078838174</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.6919999999999999</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.7361702127659574</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.5640000000000001</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.484</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.5105485232067511</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.5394190871369295</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.5559999999999999</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.5864978902953586</v>
       </c>
     </row>
   </sheetData>
@@ -1078,7 +2464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1121,7 +2507,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>tiny-aya-earth</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1133,22 +2519,22 @@
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>0.752</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>0.748</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="F2" t="n">
         <v>0.004</v>
       </c>
       <c r="G2" t="n">
-        <v>0.744</v>
+        <v>0.6840000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>tiny-aya-earth</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1163,19 +2549,19 @@
         <v>0.592</v>
       </c>
       <c r="E3" t="n">
-        <v>0.58</v>
+        <v>0.572</v>
       </c>
       <c r="F3" t="n">
-        <v>0.012</v>
+        <v>0.02</v>
       </c>
       <c r="G3" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.552</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>tiny-aya-earth</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1187,22 +2573,22 @@
         <v>250</v>
       </c>
       <c r="D4" t="n">
-        <v>0.54</v>
+        <v>0.572</v>
       </c>
       <c r="E4" t="n">
-        <v>0.536</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>0.004</v>
+        <v>0.012</v>
       </c>
       <c r="G4" t="n">
-        <v>0.532</v>
+        <v>0.548</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>tiny-aya-global</t>
+          <t>tiny-aya-earth</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1214,43 +2600,448 @@
         <v>250</v>
       </c>
       <c r="D5" t="n">
-        <v>0.536</v>
+        <v>0.532</v>
       </c>
       <c r="E5" t="n">
-        <v>0.524</v>
+        <v>0.516</v>
       </c>
       <c r="F5" t="n">
-        <v>0.012</v>
+        <v>0.016</v>
       </c>
       <c r="G5" t="n">
-        <v>0.512</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>tiny-aya-earth</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>250</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.584</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.576</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.5679999999999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>250</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.672</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.668</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>250</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.556</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>250</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.528</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.512</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>250</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.544</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.528</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.512</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>tiny-aya-fire</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>250</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.576</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.5639999999999999</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.552</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>tiny-aya-global</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>250</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.752</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.748</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.744</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>250</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.592</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.5679999999999999</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>250</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.532</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>250</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.524</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.512</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>tiny-aya-global</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>sw</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>250</v>
-      </c>
-      <c r="D6" t="n">
+      <c r="C16" t="n">
+        <v>250</v>
+      </c>
+      <c r="D16" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E16" t="n">
         <v>0.556</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F16" t="n">
         <v>0.004</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G16" t="n">
         <v>0.552</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>250</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.6919999999999999</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.6919999999999999</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.6919999999999999</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>zh</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>250</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.588</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.576</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.5639999999999999</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>bn</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>250</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.516</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.484</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>te</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>250</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.544</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.532</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.52</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>tiny-aya-water</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>250</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.556</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.556</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>